<commit_message>
Update the excel sheet
</commit_message>
<xml_diff>
--- a/March.xlsx
+++ b/March.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramji/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramji/Desktop/nConnect Feb Analytics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA35FC4A-3FD3-704C-836C-463DCF7D2E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC11472-62A2-5342-8BB7-A282FA5F54F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3929,7 +3929,9 @@
       <c r="E58" s="8">
         <v>46086</v>
       </c>
-      <c r="F58" s="7"/>
+      <c r="F58" s="8">
+        <v>46128</v>
+      </c>
       <c r="G58" s="12" t="s">
         <v>182</v>
       </c>
@@ -3975,7 +3977,9 @@
       <c r="E59" s="8">
         <v>46086</v>
       </c>
-      <c r="F59" s="7"/>
+      <c r="F59" s="8">
+        <v>46128</v>
+      </c>
       <c r="G59" s="12" t="s">
         <v>186</v>
       </c>
@@ -4021,7 +4025,9 @@
       <c r="E60" s="8">
         <v>46086</v>
       </c>
-      <c r="F60" s="7"/>
+      <c r="F60" s="8">
+        <v>46128</v>
+      </c>
       <c r="G60" s="7"/>
       <c r="H60" s="9" t="s">
         <v>190</v>
@@ -4065,7 +4071,9 @@
       <c r="E61" s="8">
         <v>46086</v>
       </c>
-      <c r="F61" s="7"/>
+      <c r="F61" s="8">
+        <v>46128</v>
+      </c>
       <c r="G61" s="7"/>
       <c r="H61" s="9" t="s">
         <v>193</v>
@@ -4109,7 +4117,9 @@
       <c r="E62" s="8">
         <v>46087</v>
       </c>
-      <c r="F62" s="7"/>
+      <c r="F62" s="8">
+        <v>46128</v>
+      </c>
       <c r="G62" s="12" t="s">
         <v>195</v>
       </c>
@@ -4153,7 +4163,9 @@
       <c r="E63" s="8">
         <v>46087</v>
       </c>
-      <c r="F63" s="7"/>
+      <c r="F63" s="8">
+        <v>46128</v>
+      </c>
       <c r="G63" s="7"/>
       <c r="H63" s="9" t="s">
         <v>197</v>
@@ -4197,7 +4209,9 @@
       <c r="E64" s="8">
         <v>46087</v>
       </c>
-      <c r="F64" s="7"/>
+      <c r="F64" s="8">
+        <v>46128</v>
+      </c>
       <c r="G64" s="7"/>
       <c r="H64" s="9" t="s">
         <v>200</v>
@@ -4241,7 +4255,9 @@
       <c r="E65" s="8">
         <v>46099</v>
       </c>
-      <c r="F65" s="7"/>
+      <c r="F65" s="8">
+        <v>46128</v>
+      </c>
       <c r="G65" s="7"/>
       <c r="H65" s="13" t="s">
         <v>202</v>
@@ -4285,7 +4301,9 @@
       <c r="E66" s="8">
         <v>46106</v>
       </c>
-      <c r="F66" s="7"/>
+      <c r="F66" s="8">
+        <v>46128</v>
+      </c>
       <c r="G66" s="7"/>
       <c r="H66" s="9" t="s">
         <v>205</v>
@@ -4329,7 +4347,9 @@
       <c r="E67" s="8">
         <v>46107</v>
       </c>
-      <c r="F67" s="7"/>
+      <c r="F67" s="8">
+        <v>46128</v>
+      </c>
       <c r="G67" s="7"/>
       <c r="H67" s="9" t="s">
         <v>207</v>
@@ -4373,7 +4393,9 @@
       <c r="E68" s="8">
         <v>46107</v>
       </c>
-      <c r="F68" s="7"/>
+      <c r="F68" s="8">
+        <v>46128</v>
+      </c>
       <c r="G68" s="7"/>
       <c r="H68" s="9" t="s">
         <v>210</v>
@@ -4417,7 +4439,9 @@
       <c r="E69" s="8">
         <v>46107</v>
       </c>
-      <c r="F69" s="7"/>
+      <c r="F69" s="8">
+        <v>46128</v>
+      </c>
       <c r="G69" s="7"/>
       <c r="H69" s="9" t="s">
         <v>212</v>
@@ -4461,7 +4485,9 @@
       <c r="E70" s="8">
         <v>46108</v>
       </c>
-      <c r="F70" s="7"/>
+      <c r="F70" s="8">
+        <v>46128</v>
+      </c>
       <c r="G70" s="7"/>
       <c r="H70" s="14" t="s">
         <v>215</v>
@@ -4505,7 +4531,9 @@
       <c r="E71" s="8">
         <v>46111</v>
       </c>
-      <c r="F71" s="7"/>
+      <c r="F71" s="8">
+        <v>46128</v>
+      </c>
       <c r="G71" s="7"/>
       <c r="H71" s="14" t="s">
         <v>218</v>
@@ -4549,7 +4577,9 @@
       <c r="E72" s="8">
         <v>46111</v>
       </c>
-      <c r="F72" s="7"/>
+      <c r="F72" s="8">
+        <v>46128</v>
+      </c>
       <c r="G72" s="7"/>
       <c r="H72" s="14" t="s">
         <v>221</v>

</xml_diff>